<commit_message>
Oprava cennika: 5 realnych materialov z konfiguratora (Premiova syntet. koza + Mikrosemis)
</commit_message>
<xml_diff>
--- a/cennik_konfigurator.xlsx
+++ b/cennik_konfigurator.xlsx
@@ -13,17 +13,19 @@
     <sheet name="Scenáre zákazníkov" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="MAT_ALCANTARA" vbProcedure="false">Cenník!$B$11</definedName>
-    <definedName function="false" hidden="false" name="MAT_EKOKOZA" vbProcedure="false">Cenník!$B$10</definedName>
-    <definedName function="false" hidden="false" name="MAT_PRESIVANA" vbProcedure="false">Cenník!$B$12</definedName>
-    <definedName function="false" hidden="false" name="NAS_BOKY" vbProcedure="false">Cenník!$B$22</definedName>
-    <definedName function="false" hidden="false" name="NAS_BOKY_SAMO" vbProcedure="false">Cenník!$C$22</definedName>
-    <definedName function="false" hidden="false" name="NAS_BUNDLE" vbProcedure="false">Cenník!$B$23</definedName>
-    <definedName function="false" hidden="false" name="NAS_DVERE" vbProcedure="false">Cenník!$B$39</definedName>
-    <definedName function="false" hidden="false" name="NAS_STRED" vbProcedure="false">Cenník!$B$21</definedName>
-    <definedName function="false" hidden="false" name="NAS_STRED_SAMO" vbProcedure="false">Cenník!$C$21</definedName>
-    <definedName function="false" hidden="false" name="TAPACIR_BUNDLE" vbProcedure="false">Cenník!$B$31</definedName>
-    <definedName function="false" hidden="false" name="TAPACIR_SAMO" vbProcedure="false">Cenník!$C$31</definedName>
+    <definedName function="false" hidden="false" name="MAT_KOZA_JEDNO" vbProcedure="false">Cenník!$B$10</definedName>
+    <definedName function="false" hidden="false" name="MAT_KOZA_PRESIV" vbProcedure="false">Cenník!$B$11</definedName>
+    <definedName function="false" hidden="false" name="MAT_KOZA_TONOV" vbProcedure="false">Cenník!$B$12</definedName>
+    <definedName function="false" hidden="false" name="MAT_MIKRO_DVOJ" vbProcedure="false">Cenník!$B$14</definedName>
+    <definedName function="false" hidden="false" name="MAT_MIKRO_JEDNO" vbProcedure="false">Cenník!$B$13</definedName>
+    <definedName function="false" hidden="false" name="NAS_BOKY" vbProcedure="false">Cenník!$B$24</definedName>
+    <definedName function="false" hidden="false" name="NAS_BOKY_SAMO" vbProcedure="false">Cenník!$C$24</definedName>
+    <definedName function="false" hidden="false" name="NAS_BUNDLE" vbProcedure="false">Cenník!$B$25</definedName>
+    <definedName function="false" hidden="false" name="NAS_DVERE" vbProcedure="false">Cenník!$B$41</definedName>
+    <definedName function="false" hidden="false" name="NAS_STRED" vbProcedure="false">Cenník!$B$23</definedName>
+    <definedName function="false" hidden="false" name="NAS_STRED_SAMO" vbProcedure="false">Cenník!$C$23</definedName>
+    <definedName function="false" hidden="false" name="TAPACIR_BUNDLE" vbProcedure="false">Cenník!$B$33</definedName>
+    <definedName function="false" hidden="false" name="TAPACIR_SAMO" vbProcedure="false">Cenník!$C$33</definedName>
     <definedName function="false" hidden="false" name="ZAKLAD" vbProcedure="false">Cenník!$B$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -36,12 +38,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="107">
   <si>
     <t xml:space="preserve">KONFIGURÁTOR KAMIÓNOV — CENNÍK</t>
   </si>
   <si>
-    <t xml:space="preserve">Modré bunky = editovateľné ceny · Zelené = bundle cena (úspora) · LUXURY CAR DESIGN</t>
+    <t xml:space="preserve">Modré = editovateľné ceny · Zelené = bundle cena (úspora) · LUXURY CAR DESIGN</t>
   </si>
   <si>
     <t xml:space="preserve">Položka</t>
@@ -71,22 +73,34 @@
     <t xml:space="preserve">BOD 2 — MATERIÁL (len druh mení cenu, farba NIE)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ekokoža (štandard)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">V cene základu — bez príplatku</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcantara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Príplatok k základu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prešívaná koža</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prémiový príplatok</t>
+    <t xml:space="preserve">Prémiová syntetická koža – jednofarebná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Základ — bez príplatku</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prémiová syntetická koža – prešívaná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Príplatok — prešívaný povrch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prémiová syntetická koža – tónovaná</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Príplatok — tónovaný vzhľad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mikrosemiš – jednofarebný</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Príplatok — jemný povrch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mikrosemiš – dvojfarebný</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Príplatok — dvojfarebný efekt</t>
   </si>
   <si>
     <t xml:space="preserve">Farba materiálu</t>
@@ -104,7 +118,7 @@
     <t xml:space="preserve">V cene základu — zákazník vyberá bez príplatku</t>
   </si>
   <si>
-    <t xml:space="preserve">BOD 4 — NÁŠIVKY (bod 4a mení cenu, bod 4b, 4c NIE)</t>
+    <t xml:space="preserve">BOD 4 — NÁŠIVKY (bod 4a mení cenu, 4b/4c NIE)</t>
   </si>
   <si>
     <t xml:space="preserve">4a — UMIESTNENIE NÁŠIVIEK</t>
@@ -113,7 +127,7 @@
     <t xml:space="preserve">Bez nášiviek</t>
   </si>
   <si>
-    <t xml:space="preserve">Zákazník nechce nášivky — NEMENÍ cenu</t>
+    <t xml:space="preserve">NEMENÍ cenu</t>
   </si>
   <si>
     <t xml:space="preserve">Len stred (samostatne)</t>
@@ -140,7 +154,7 @@
     <t xml:space="preserve">Výber druhu nášivky a farby nite</t>
   </si>
   <si>
-    <t xml:space="preserve">Všetky druhy nášiviek a farieb v cene — NEMENÍ cenu</t>
+    <t xml:space="preserve">Všetky druhy nášiviek a farieb v cene</t>
   </si>
   <si>
     <t xml:space="preserve">BOD 5 — TAPACÍR DVERÍ</t>
@@ -176,19 +190,16 @@
     <t xml:space="preserve">Lemovanie tapacíra</t>
   </si>
   <si>
-    <t xml:space="preserve">5d — NÁŠIVKA NA DVEREÁCH (áno = príplatok)</t>
+    <t xml:space="preserve">5d — NÁŠIVKA NA DVERÁCH (áno = príplatok)</t>
   </si>
   <si>
     <t xml:space="preserve">Nie nechcem nášivku na dverách</t>
   </si>
   <si>
-    <t xml:space="preserve">NEMENÍ cenu</t>
-  </si>
-  <si>
     <t xml:space="preserve">Áno chcem nášivku na dverách</t>
   </si>
   <si>
-    <t xml:space="preserve">Príplatok za nášivku na tapacíri dverí (vzorová cena — uprav podľa potreby)</t>
+    <t xml:space="preserve">Príplatok za nášivku na tapacíri (vzorová cena — uprav podľa potreby)</t>
   </si>
   <si>
     <t xml:space="preserve">LEGENDA FARIEB</t>
@@ -239,16 +250,7 @@
     <t xml:space="preserve">BOD 2 — Materiál</t>
   </si>
   <si>
-    <t xml:space="preserve">Vyber druh materiálu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOD 2 — Farba materiálu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ľubovoľná</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Farba NEMENÍ cenu</t>
+    <t xml:space="preserve">Vyber druh materiálu (farba NEMENÍ cenu)</t>
   </si>
   <si>
     <t xml:space="preserve">BOD 3 — Lemovanie</t>
@@ -293,7 +295,7 @@
     <t xml:space="preserve">Hypotetická cena mimo konfigurátora</t>
   </si>
   <si>
-    <t xml:space="preserve">Súčet samostatných cien (keď platí stĺpec C v cenníku)</t>
+    <t xml:space="preserve">Súčet samostatných cien</t>
   </si>
   <si>
     <t xml:space="preserve">TVOJA CENA V KONFIGURÁTORE</t>
@@ -324,9 +326,6 @@
   </si>
   <si>
     <t xml:space="preserve">Materiál</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ekokoža</t>
   </si>
   <si>
     <t xml:space="preserve">Nášivky (4a)</t>
@@ -371,7 +370,7 @@
     <numFmt numFmtId="165" formatCode="#,##0&quot; €&quot;;[RED]\-#,##0&quot; €&quot;;\—"/>
     <numFmt numFmtId="166" formatCode="0%;\-0%;\—"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -489,14 +488,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
@@ -712,23 +703,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -740,11 +727,11 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -756,8 +743,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -768,16 +763,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1032,13 +1023,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1076,6 +1067,7 @@
         <v>6</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>7</v>
@@ -1126,7 +1118,7 @@
         <v>13</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8"/>
@@ -1139,7 +1131,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8"/>
@@ -1152,7 +1144,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8"/>
@@ -1160,208 +1152,212 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
+      <c r="B14" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="9" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="B15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-    </row>
-    <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="9" t="s">
+      <c r="B18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="9" t="s">
         <v>25</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+    </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="C21" s="7" t="n">
-        <v>70</v>
-      </c>
-      <c r="D21" s="8"/>
-      <c r="E21" s="9" t="s">
+      <c r="A21" s="10" t="s">
         <v>27</v>
       </c>
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
         <v>28</v>
       </c>
       <c r="B22" s="6" t="n">
-        <v>70</v>
-      </c>
-      <c r="C22" s="7" t="n">
-        <v>70</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C22" s="7"/>
       <c r="D22" s="8"/>
       <c r="E22" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D23" s="8"/>
+      <c r="E23" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="C24" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D24" s="8"/>
+      <c r="E24" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="C23" s="13" t="n">
+      <c r="C25" s="13" t="n">
         <v>140</v>
       </c>
-      <c r="D23" s="14" t="n">
-        <f aca="false">IF(AND(B23&gt;0,C23&gt;0),1-B23/C23,0)</f>
+      <c r="D25" s="14" t="n">
+        <f aca="false">IF(AND(B25&gt;0,C25&gt;0),1-B25/C25,0)</f>
         <v>0.285714285714286</v>
       </c>
-      <c r="E23" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="E25" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-    </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
+    </row>
+    <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-    </row>
-    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="7"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="9" t="s">
+      <c r="B28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="9" t="s">
         <v>38</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="30" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+    </row>
     <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="12" t="n">
+      <c r="A31" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="C31" s="13" t="n">
+      <c r="C33" s="13" t="n">
         <v>179</v>
       </c>
-      <c r="D31" s="14" t="n">
-        <f aca="false">IF(AND(B31&gt;0,C31&gt;0),1-B31/C31,0)</f>
+      <c r="D33" s="14" t="n">
+        <f aca="false">IF(AND(B33&gt;0,C33&gt;0),1-B33/C33,0)</f>
         <v>0.441340782122905</v>
       </c>
-      <c r="E31" s="15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-    </row>
-    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="9" t="s">
-        <v>43</v>
-      </c>
-    </row>
+      <c r="E33" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -1370,7 +1366,7 @@
     </row>
     <row r="36" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B36" s="6" t="n">
         <v>0</v>
@@ -1378,12 +1374,12 @@
       <c r="C36" s="7"/>
       <c r="D36" s="8"/>
       <c r="E36" s="9" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -1392,7 +1388,7 @@
     </row>
     <row r="38" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B38" s="6" t="n">
         <v>0</v>
@@ -1400,66 +1396,88 @@
       <c r="C38" s="7"/>
       <c r="D38" s="8"/>
       <c r="E38" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" s="6" t="n">
+      <c r="A39" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="C39" s="7" t="n">
+      <c r="B39" s="10"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+    </row>
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="7"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="D39" s="8"/>
-      <c r="E39" s="9" t="s">
+      <c r="C41" s="7" t="n">
         <v>50</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
-      <c r="D41" s="16"/>
-      <c r="E41" s="16"/>
-    </row>
-    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B42" s="18" t="s">
+      <c r="D41" s="8"/>
+      <c r="E41" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-    </row>
+    </row>
+    <row r="42" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="43" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="s">
+      <c r="A43" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B43" s="18" t="s">
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+    </row>
+    <row r="44" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C43" s="18"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-    </row>
-    <row r="44" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="20" t="s">
+      <c r="B44" s="18" t="s">
         <v>56</v>
-      </c>
-      <c r="B44" s="18" t="s">
-        <v>57</v>
       </c>
       <c r="C44" s="18"/>
       <c r="D44" s="18"/>
       <c r="E44" s="18"/>
+    </row>
+    <row r="45" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C46" s="18"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -1467,19 +1485,19 @@
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A30:E30"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A35:E35"/>
     <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B43:E43"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A43:E43"/>
     <mergeCell ref="B44:E44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1496,18 +1514,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1515,7 +1533,7 @@
     </row>
     <row r="2" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1523,13 +1541,13 @@
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>6</v>
@@ -1537,194 +1555,180 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C5" s="23" t="n">
         <f aca="false">ZAKLAD</f>
         <v>200</v>
       </c>
-      <c r="D5" s="24" t="s">
-        <v>65</v>
+      <c r="D5" s="22" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="B6" s="26" t="s">
+      <c r="A6" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="27" t="n">
-        <f aca="false">IF(B6="Ekokoža (štandard)",MAT_EKOKOZA,IF(B6="Alcantara",MAT_ALCANTARA,IF(B6="Prešívaná koža",MAT_PRESIVANA,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>67</v>
+      <c r="C6" s="26" t="n">
+        <f aca="false">IF(B6="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(B6="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(B6="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(B6="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(B6="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B7" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>70</v>
+      <c r="A7" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="26" t="s">
+      <c r="A8" s="24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="26" t="n">
+        <f aca="false">IF(B8="Bez nášiviek",0,IF(B8="Len stred",NAS_STRED,IF(B8="Šofér + spolujazdec",NAS_BOKY,IF(B8="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="27" t="str">
+        <f aca="false">IF(B8="Šofér + spolujazdec + stred (BUNDLE)","✓ Ušetríte "&amp;TEXT(NAS_BOKY_SAMO+NAS_STRED_SAMO-NAS_BUNDLE,"0")&amp;" € oproti samostatnému výberu!","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="27" t="n">
-        <f aca="false">IF(B9="Bez nášiviek",0,IF(B9="Len stred",NAS_STRED,IF(B9="Šofér + spolujazdec",NAS_BOKY,IF(B9="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))</f>
-        <v>0</v>
-      </c>
-      <c r="D9" s="28" t="str">
-        <f aca="false">IF(B9="Šofér + spolujazdec + stred (BUNDLE)","✓ Ušetríte "&amp;TEXT(NAS_BOKY_SAMO+NAS_STRED_SAMO-NAS_BUNDLE,"0")&amp;" € oproti samostatnému výberu!","")</f>
+      <c r="C9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="26" t="n">
+        <f aca="false">IF(B10="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="27" t="str">
+        <f aca="false">IF(B10="Áno chcem (v konfigurátore)","✓ Bežne "&amp;TEXT(TAPACIR_SAMO,"0")&amp;" €, ušetríte "&amp;TEXT(TAPACIR_SAMO-TAPACIR_BUNDLE,"0")&amp;" €!","")</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="26" t="s">
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="26" t="s">
+      <c r="C11" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="27" t="n">
-        <f aca="false">IF(B11="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D11" s="28" t="str">
-        <f aca="false">IF(B11="Áno chcem (v konfigurátore)","✓ Bežne "&amp;TEXT(TAPACIR_SAMO,"0")&amp;" €, ušetríte "&amp;TEXT(TAPACIR_SAMO-TAPACIR_BUNDLE,"0")&amp;" €!","")</f>
+      <c r="C12" s="26" t="n">
+        <f aca="false">IF(B12="Áno chcem",NAS_DVERE,0)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="27" t="str">
+        <f aca="false">IF(B12="Áno chcem","Príplatok za nášivku na dverách","")</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B13" s="26" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="27" t="n">
-        <f aca="false">IF(B13="Áno chcem",NAS_DVERE,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D13" s="28" t="str">
-        <f aca="false">IF(B13="Áno chcem","Príplatok za nášivku na dverách","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="29" t="s">
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28" t="s">
         <v>81</v>
       </c>
-      <c r="B15" s="29"/>
-      <c r="C15" s="30" t="n">
-        <f aca="false">SUM(C5:C13)</f>
+      <c r="B14" s="28"/>
+      <c r="C14" s="29" t="n">
+        <f aca="false">SUM(C5:C12)</f>
         <v>200</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D14" s="30" t="s">
         <v>82</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+    </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="A17" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="31"/>
+      <c r="C17" s="32" t="n">
+        <f aca="false">ZAKLAD+IF(B6="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(B6="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(B6="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(B6="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(B6="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(B8="Bez nášiviek",0,IF(B8="Len stred",NAS_STRED_SAMO,IF(B8="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(B8="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(B10="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(B12="Áno chcem",NAS_DVERE,0)</f>
+        <v>200</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="27" t="n">
-        <f aca="false">ZAKLAD+IF(B6="Ekokoža (štandard)",MAT_EKOKOZA,IF(B6="Alcantara",MAT_ALCANTARA,IF(B6="Prešívaná koža",MAT_PRESIVANA,0)))+IF(B9="Bez nášiviek",0,IF(B9="Len stred",NAS_STRED_SAMO,IF(B9="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(B9="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(B11="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(B13="Áno chcem",NAS_DVERE,0)</f>
+      <c r="A18" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="32" t="n">
+        <f aca="false">C14</f>
         <v>200</v>
       </c>
-      <c r="D18" s="32" t="s">
-        <v>85</v>
-      </c>
+      <c r="D18" s="31"/>
     </row>
     <row r="19" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="33" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="27" t="n">
-        <f aca="false">C15</f>
-        <v>200</v>
-      </c>
-      <c r="D19" s="32"/>
-    </row>
-    <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="33" t="s">
         <v>87</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="27" t="n">
-        <f aca="false">C18-C15</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="34" t="str">
-        <f aca="false">IF(C18&gt;0,"= "&amp;TEXT((C18-C15)/C18,"0%")&amp;" zľava oproti mimokonfigurátorovej cene","")</f>
+      <c r="B19" s="31"/>
+      <c r="C19" s="34" t="n">
+        <f aca="false">C17-C14</f>
+        <v>0</v>
+      </c>
+      <c r="D19" s="35" t="str">
+        <f aca="false">IF(C17&gt;0,"= "&amp;TEXT((C17-C14)/C17,"0%")&amp;" zľava oproti mimokonfigurátorovej cene","")</f>
         <v>= 0% zľava oproti mimokonfigurátorovej cene</v>
       </c>
     </row>
@@ -1732,23 +1736,23 @@
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B6" type="list">
-      <formula1>"Ekokoža (štandard),Alcantara,Prešívaná koža"</formula1>
+      <formula1>"Prémiová syntetická koža – jednofarebná,Prémiová syntetická koža – prešívaná,Prémiová syntetická koža – tónovaná,Mikrosemiš – jednofarebný,Mikrosemiš – dvojfarebný"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B9" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B8" type="list">
       <formula1>"Bez nášiviek,Len stred,Šofér + spolujazdec,Šofér + spolujazdec + stred (BUNDLE)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B11" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B10" type="list">
       <formula1>"Nie nechcem,Áno chcem (v konfigurátore)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B13" type="list">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B12" type="list">
       <formula1>"Nie nechcem,Áno chcem"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1771,8 +1775,8 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1783,8 +1787,9 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>89</v>
       </c>
@@ -1804,165 +1809,165 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
+    <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B4" s="35" t="s">
+      <c r="B4" s="36" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="36" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="36" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
         <v>96</v>
       </c>
-      <c r="C4" s="35" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
+      <c r="B5" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="36" t="s">
         <v>97</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="35" t="s">
+      <c r="D5" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="E5" s="36" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" s="36" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E5" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="35" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
+      <c r="B6" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" s="36" t="s">
         <v>100</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="F6" s="36" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="35" t="s">
+      <c r="C7" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D7" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="F6" s="35" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
+      <c r="E7" s="36" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="B7" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="D7" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="E7" s="35" t="s">
-        <v>78</v>
-      </c>
-      <c r="F7" s="35" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
+      <c r="B9" s="37" t="n">
+        <f aca="false">ZAKLAD+IF(B4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(B4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(B4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(B4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(B4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(B5="Bez nášiviek",0,IF(B5="Len stred",NAS_STRED,IF(B5="Šofér + spolujazdec",NAS_BOKY,IF(B5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(B6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(B7="Áno chcem",NAS_DVERE,0)</f>
+        <v>200</v>
+      </c>
+      <c r="C9" s="37" t="n">
+        <f aca="false">ZAKLAD+IF(C4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(C4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(C4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(C4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(C4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(C5="Bez nášiviek",0,IF(C5="Len stred",NAS_STRED,IF(C5="Šofér + spolujazdec",NAS_BOKY,IF(C5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(C6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(C7="Áno chcem",NAS_DVERE,0)</f>
+        <v>270</v>
+      </c>
+      <c r="D9" s="37" t="n">
+        <f aca="false">ZAKLAD+IF(D4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(D4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(D4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(D4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(D4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(D5="Bez nášiviek",0,IF(D5="Len stred",NAS_STRED,IF(D5="Šofér + spolujazdec",NAS_BOKY,IF(D5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(D6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(D7="Áno chcem",NAS_DVERE,0)</f>
+        <v>290</v>
+      </c>
+      <c r="E9" s="37" t="n">
+        <f aca="false">ZAKLAD+IF(E4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(E4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(E4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(E4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(E4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(E5="Bez nášiviek",0,IF(E5="Len stred",NAS_STRED,IF(E5="Šofér + spolujazdec",NAS_BOKY,IF(E5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(E6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(E7="Áno chcem",NAS_DVERE,0)</f>
+        <v>430</v>
+      </c>
+      <c r="F9" s="37" t="n">
+        <f aca="false">ZAKLAD+IF(F4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(F4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(F4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(F4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(F4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(F5="Bez nášiviek",0,IF(F5="Len stred",NAS_STRED,IF(F5="Šofér + spolujazdec",NAS_BOKY,IF(F5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(F6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(F7="Áno chcem",NAS_DVERE,0)</f>
+        <v>490</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="B9" s="36" t="n">
-        <f aca="false">ZAKLAD+IF(B4="Ekokoža",MAT_EKOKOZA,IF(B4="Alcantara",MAT_ALCANTARA,IF(B4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(B5="Bez nášiviek",0,IF(B5="Len stred",NAS_STRED,IF(B5="Šofér + spolujazdec",NAS_BOKY,IF(B5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(B6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(B7="Áno chcem",NAS_DVERE,0)</f>
+      <c r="B10" s="7" t="n">
+        <f aca="false">ZAKLAD+IF(B4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(B4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(B4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(B4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(B4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(B5="Bez nášiviek",0,IF(B5="Len stred",NAS_STRED_SAMO,IF(B5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(B5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(B6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(B7="Áno chcem",NAS_DVERE,0)</f>
         <v>200</v>
       </c>
-      <c r="C9" s="36" t="n">
-        <f aca="false">ZAKLAD+IF(C4="Ekokoža",MAT_EKOKOZA,IF(C4="Alcantara",MAT_ALCANTARA,IF(C4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(C5="Bez nášiviek",0,IF(C5="Len stred",NAS_STRED,IF(C5="Šofér + spolujazdec",NAS_BOKY,IF(C5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(C6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(C7="Áno chcem",NAS_DVERE,0)</f>
+      <c r="C10" s="7" t="n">
+        <f aca="false">ZAKLAD+IF(C4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(C4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(C4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(C4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(C4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(C5="Bez nášiviek",0,IF(C5="Len stred",NAS_STRED_SAMO,IF(C5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(C5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(C6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(C7="Áno chcem",NAS_DVERE,0)</f>
         <v>270</v>
       </c>
-      <c r="D9" s="36" t="n">
-        <f aca="false">ZAKLAD+IF(D4="Ekokoža",MAT_EKOKOZA,IF(D4="Alcantara",MAT_ALCANTARA,IF(D4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(D5="Bez nášiviek",0,IF(D5="Len stred",NAS_STRED,IF(D5="Šofér + spolujazdec",NAS_BOKY,IF(D5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(D6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(D7="Áno chcem",NAS_DVERE,0)</f>
-        <v>300</v>
-      </c>
-      <c r="E9" s="36" t="n">
-        <f aca="false">ZAKLAD+IF(E4="Ekokoža",MAT_EKOKOZA,IF(E4="Alcantara",MAT_ALCANTARA,IF(E4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(E5="Bez nášiviek",0,IF(E5="Len stred",NAS_STRED,IF(E5="Šofér + spolujazdec",NAS_BOKY,IF(E5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(E6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(E7="Áno chcem",NAS_DVERE,0)</f>
-        <v>430</v>
-      </c>
-      <c r="F9" s="36" t="n">
-        <f aca="false">ZAKLAD+IF(F4="Ekokoža",MAT_EKOKOZA,IF(F4="Alcantara",MAT_ALCANTARA,IF(F4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(F5="Bez nášiviek",0,IF(F5="Len stred",NAS_STRED,IF(F5="Šofér + spolujazdec",NAS_BOKY,IF(F5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BUNDLE,0))))+IF(F6="Áno chcem (v konfigurátore)",TAPACIR_BUNDLE,0)+IF(F7="Áno chcem",NAS_DVERE,0)</f>
-        <v>500</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="s">
+      <c r="D10" s="7" t="n">
+        <f aca="false">ZAKLAD+IF(D4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(D4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(D4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(D4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(D4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(D5="Bez nášiviek",0,IF(D5="Len stred",NAS_STRED_SAMO,IF(D5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(D5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(D6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(D7="Áno chcem",NAS_DVERE,0)</f>
+        <v>290</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <f aca="false">ZAKLAD+IF(E4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(E4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(E4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(E4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(E4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(E5="Bez nášiviek",0,IF(E5="Len stred",NAS_STRED_SAMO,IF(E5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(E5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(E6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(E7="Áno chcem",NAS_DVERE,0)</f>
+        <v>549</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <f aca="false">ZAKLAD+IF(F4="Prémiová syntetická koža – jednofarebná",MAT_KOZA_JEDNO,IF(F4="Prémiová syntetická koža – prešívaná",MAT_KOZA_PRESIV,IF(F4="Prémiová syntetická koža – tónovaná",MAT_KOZA_TONOV,IF(F4="Mikrosemiš – jednofarebný",MAT_MIKRO_JEDNO,IF(F4="Mikrosemiš – dvojfarebný",MAT_MIKRO_DVOJ,0)))))+IF(F5="Bez nášiviek",0,IF(F5="Len stred",NAS_STRED_SAMO,IF(F5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(F5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(F6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(F7="Áno chcem",NAS_DVERE,0)</f>
+        <v>609</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <f aca="false">ZAKLAD+IF(B4="Ekokoža",MAT_EKOKOZA,IF(B4="Alcantara",MAT_ALCANTARA,IF(B4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(B5="Bez nášiviek",0,IF(B5="Len stred",NAS_STRED_SAMO,IF(B5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(B5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(B6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(B7="Áno chcem",NAS_DVERE,0)</f>
-        <v>200</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <f aca="false">ZAKLAD+IF(C4="Ekokoža",MAT_EKOKOZA,IF(C4="Alcantara",MAT_ALCANTARA,IF(C4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(C5="Bez nášiviek",0,IF(C5="Len stred",NAS_STRED_SAMO,IF(C5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(C5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(C6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(C7="Áno chcem",NAS_DVERE,0)</f>
-        <v>270</v>
-      </c>
-      <c r="D10" s="7" t="n">
-        <f aca="false">ZAKLAD+IF(D4="Ekokoža",MAT_EKOKOZA,IF(D4="Alcantara",MAT_ALCANTARA,IF(D4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(D5="Bez nášiviek",0,IF(D5="Len stred",NAS_STRED_SAMO,IF(D5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(D5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(D6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(D7="Áno chcem",NAS_DVERE,0)</f>
-        <v>300</v>
-      </c>
-      <c r="E10" s="7" t="n">
-        <f aca="false">ZAKLAD+IF(E4="Ekokoža",MAT_EKOKOZA,IF(E4="Alcantara",MAT_ALCANTARA,IF(E4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(E5="Bez nášiviek",0,IF(E5="Len stred",NAS_STRED_SAMO,IF(E5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(E5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(E6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(E7="Áno chcem",NAS_DVERE,0)</f>
-        <v>549</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <f aca="false">ZAKLAD+IF(F4="Ekokoža",MAT_EKOKOZA,IF(F4="Alcantara",MAT_ALCANTARA,IF(F4="Prešívaná koža",MAT_PRESIVANA,0)))+IF(F5="Bez nášiviek",0,IF(F5="Len stred",NAS_STRED_SAMO,IF(F5="Šofér + spolujazdec",NAS_BOKY_SAMO,IF(F5="Šofér + spolujazdec + stred (BUNDLE)",NAS_BOKY_SAMO+NAS_STRED_SAMO,0))))+IF(F6="Áno chcem (v konfigurátore)",TAPACIR_SAMO,0)+IF(F7="Áno chcem",NAS_DVERE,0)</f>
-        <v>619</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="34" t="n">
         <f aca="false">B10-B9</f>
         <v>0</v>
       </c>
-      <c r="C11" s="38" t="n">
+      <c r="C11" s="34" t="n">
         <f aca="false">C10-C9</f>
         <v>0</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="34" t="n">
         <f aca="false">D10-D9</f>
         <v>0</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="34" t="n">
         <f aca="false">E10-E9</f>
         <v>119</v>
       </c>
-      <c r="F11" s="38" t="n">
+      <c r="F11" s="34" t="n">
         <f aca="false">F10-F9</f>
         <v>119</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
-        <v>107</v>
+    <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="27" t="s">
+        <v>106</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">IFERROR((B10-B9)/B10,0)</f>
@@ -1982,12 +1987,12 @@
       </c>
       <c r="F12" s="8" t="n">
         <f aca="false">IFERROR((F10-F9)/F10,0)</f>
-        <v>0.192245557350565</v>
+        <v>0.195402298850575</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>